<commit_message>
docs(ui): add sample excel template and download link
Adds a sample Excel file and a download link to the SMS reminder
upload view to assist users with the required file format.
</commit_message>
<xml_diff>
--- a/public/downloads/master-sample.xlsx
+++ b/public/downloads/master-sample.xlsx
@@ -1,14 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
+  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+  <workbookPr codeName="ThisWorkbook"/>
+  <bookViews>
+    <workbookView activeTab="0" autoFilterDateGrouping="true" firstSheet="0" minimized="false" showHorizontalScroll="true" showSheetTabs="true" showVerticalScroll="true" tabRatio="600" visibility="visible"/>
+  </bookViews>
   <sheets>
-    <sheet name="Master" sheetId="1" r:id="rId1"/>
+    <sheet name="Master Dataset" sheetId="1" r:id="rId4"/>
   </sheets>
+  <definedNames/>
+  <calcPr calcId="999999" calcMode="auto" calcCompleted="1" fullCalcOnLoad="0" forceFullCalc="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="24">
   <si>
     <t>RUN_DATE</t>
   </si>
@@ -50,19 +57,52 @@
   </si>
   <si>
     <t>SLT_GL_SUB_SEGMENT</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>Western</t>
+  </si>
+  <si>
+    <t>Colombo</t>
+  </si>
+  <si>
+    <t>CUST001234</t>
+  </si>
+  <si>
+    <t>Post</t>
+  </si>
+  <si>
+    <t>Residential</t>
+  </si>
+  <si>
+    <t>123, Main Street, Colombo 01</t>
+  </si>
+  <si>
+    <t>Active</t>
+  </si>
+  <si>
+    <t>FTTH</t>
+  </si>
+  <si>
+    <t>Consumer</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
+  <numFmts count="0"/>
   <fonts count="1">
     <font>
+      <b val="0"/>
+      <i val="0"/>
+      <strike val="0"/>
+      <u val="none"/>
       <sz val="11"/>
-      <color theme="1"/>
+      <color rgb="FF000000"/>
       <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="2">
@@ -86,20 +126,326 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="1">
-    <xf xfId="0"/>
+    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
+  <dxfs count="0"/>
+  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
 </styleSheet>
 </file>
 
+<file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+  <a:themeElements>
+    <a:clrScheme name="Office">
+      <a:dk1>
+        <a:sysClr val="windowText" lastClr="000000"/>
+      </a:dk1>
+      <a:lt1>
+        <a:sysClr val="window" lastClr="FFFFFF"/>
+      </a:lt1>
+      <a:dk2>
+        <a:srgbClr val="1F497D"/>
+      </a:dk2>
+      <a:lt2>
+        <a:srgbClr val="EEECE1"/>
+      </a:lt2>
+      <a:accent1>
+        <a:srgbClr val="4F81BD"/>
+      </a:accent1>
+      <a:accent2>
+        <a:srgbClr val="C0504D"/>
+      </a:accent2>
+      <a:accent3>
+        <a:srgbClr val="9BBB59"/>
+      </a:accent3>
+      <a:accent4>
+        <a:srgbClr val="8064A2"/>
+      </a:accent4>
+      <a:accent5>
+        <a:srgbClr val="4BACC6"/>
+      </a:accent5>
+      <a:accent6>
+        <a:srgbClr val="F79646"/>
+      </a:accent6>
+      <a:hlink>
+        <a:srgbClr val="0000FF"/>
+      </a:hlink>
+      <a:folHlink>
+        <a:srgbClr val="800080"/>
+      </a:folHlink>
+    </a:clrScheme>
+    <a:fontScheme name="Office">
+      <a:majorFont>
+        <a:latin typeface="Cambria"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Times New Roman"/>
+        <a:font script="Hebr" typeface="Times New Roman"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="MoolBoran"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Times New Roman"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:majorFont>
+      <a:minorFont>
+        <a:latin typeface="Calibri"/>
+        <a:ea typeface=""/>
+        <a:cs typeface=""/>
+        <a:font script="Jpan" typeface="ＭＳ Ｐゴシック"/>
+        <a:font script="Hang" typeface="맑은 고딕"/>
+        <a:font script="Hans" typeface="宋体"/>
+        <a:font script="Hant" typeface="新細明體"/>
+        <a:font script="Arab" typeface="Arial"/>
+        <a:font script="Hebr" typeface="Arial"/>
+        <a:font script="Thai" typeface="Tahoma"/>
+        <a:font script="Ethi" typeface="Nyala"/>
+        <a:font script="Beng" typeface="Vrinda"/>
+        <a:font script="Gujr" typeface="Shruti"/>
+        <a:font script="Khmr" typeface="DaunPenh"/>
+        <a:font script="Knda" typeface="Tunga"/>
+        <a:font script="Guru" typeface="Raavi"/>
+        <a:font script="Cans" typeface="Euphemia"/>
+        <a:font script="Cher" typeface="Plantagenet Cherokee"/>
+        <a:font script="Yiii" typeface="Microsoft Yi Baiti"/>
+        <a:font script="Tibt" typeface="Microsoft Himalaya"/>
+        <a:font script="Thaa" typeface="MV Boli"/>
+        <a:font script="Deva" typeface="Mangal"/>
+        <a:font script="Telu" typeface="Gautami"/>
+        <a:font script="Taml" typeface="Latha"/>
+        <a:font script="Syrc" typeface="Estrangelo Edessa"/>
+        <a:font script="Orya" typeface="Kalinga"/>
+        <a:font script="Mlym" typeface="Kartika"/>
+        <a:font script="Laoo" typeface="DokChampa"/>
+        <a:font script="Sinh" typeface="Iskoola Pota"/>
+        <a:font script="Mong" typeface="Mongolian Baiti"/>
+        <a:font script="Viet" typeface="Arial"/>
+        <a:font script="Uigh" typeface="Microsoft Uighur"/>
+        <a:font script="Geor" typeface="Sylfaen"/>
+      </a:minorFont>
+    </a:fontScheme>
+    <a:fmtScheme name="Office">
+      <a:fillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="50000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="35000">
+              <a:schemeClr val="phClr">
+                <a:tint val="37000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:tint val="15000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="1"/>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:shade val="51000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="80000">
+              <a:schemeClr val="phClr">
+                <a:shade val="93000"/>
+                <a:satMod val="130000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="94000"/>
+                <a:satMod val="135000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:lin ang="16200000" scaled="0"/>
+        </a:gradFill>
+      </a:fillStyleLst>
+      <a:lnStyleLst>
+        <a:ln w="9525" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr">
+              <a:shade val="95000"/>
+              <a:satMod val="105000"/>
+            </a:schemeClr>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="25400" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+        <a:ln w="38100" cap="flat" cmpd="sng" algn="ctr">
+          <a:solidFill>
+            <a:schemeClr val="phClr"/>
+          </a:solidFill>
+          <a:prstDash val="solid"/>
+        </a:ln>
+      </a:lnStyleLst>
+      <a:effectStyleLst>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="20000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="38000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+        </a:effectStyle>
+        <a:effectStyle>
+          <a:effectLst>
+            <a:outerShdw blurRad="40000" dist="23000" dir="5400000" rotWithShape="0">
+              <a:srgbClr val="000000">
+                <a:alpha val="35000"/>
+              </a:srgbClr>
+            </a:outerShdw>
+          </a:effectLst>
+          <a:scene3d>
+            <a:camera prst="orthographicFront">
+              <a:rot lat="0" lon="0" rev="0"/>
+            </a:camera>
+            <a:lightRig rig="threePt" dir="t">
+              <a:rot lat="0" lon="0" rev="1200000"/>
+            </a:lightRig>
+          </a:scene3d>
+          <a:sp3d>
+            <a:bevelT w="63500" h="25400"/>
+          </a:sp3d>
+        </a:effectStyle>
+      </a:effectStyleLst>
+      <a:bgFillStyleLst>
+        <a:solidFill>
+          <a:schemeClr val="phClr"/>
+        </a:solidFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="40000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="40000">
+              <a:schemeClr val="phClr">
+                <a:tint val="45000"/>
+                <a:shade val="99000"/>
+                <a:satMod val="350000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="20000"/>
+                <a:satMod val="255000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="-80000" r="50000" b="180000"/>
+          </a:path>
+        </a:gradFill>
+        <a:gradFill rotWithShape="1">
+          <a:gsLst>
+            <a:gs pos="0">
+              <a:schemeClr val="phClr">
+                <a:tint val="80000"/>
+                <a:satMod val="300000"/>
+              </a:schemeClr>
+            </a:gs>
+            <a:gs pos="100000">
+              <a:schemeClr val="phClr">
+                <a:shade val="30000"/>
+                <a:satMod val="200000"/>
+              </a:schemeClr>
+            </a:gs>
+          </a:gsLst>
+          <a:path path="circle">
+            <a:fillToRect l="50000" t="50000" r="50000" b="50000"/>
+          </a:path>
+        </a:gradFill>
+      </a:bgFillStyleLst>
+    </a:fmtScheme>
+  </a:themeElements>
+  <a:objectDefaults/>
+  <a:extraClrSchemeLst/>
+</a:theme>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:N1"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xml:space="preserve" mc:Ignorable="x14ac">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+  </sheetPr>
+  <dimension ref="A1:N2"/>
+  <sheetFormatPr defaultRowHeight="14.4" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col min="1" max="1" width="22" customWidth="true" style="0"/>
+    <col min="2" max="2" width="22" customWidth="true" style="0"/>
+    <col min="3" max="3" width="22" customWidth="true" style="0"/>
+    <col min="4" max="4" width="22" customWidth="true" style="0"/>
+    <col min="5" max="5" width="22" customWidth="true" style="0"/>
+    <col min="6" max="6" width="22" customWidth="true" style="0"/>
+    <col min="7" max="7" width="22" customWidth="true" style="0"/>
+    <col min="8" max="8" width="22" customWidth="true" style="0"/>
+    <col min="9" max="9" width="22" customWidth="true" style="0"/>
+    <col min="10" max="10" width="22" customWidth="true" style="0"/>
+    <col min="11" max="11" width="22" customWidth="true" style="0"/>
+    <col min="12" max="12" width="22" customWidth="true" style="0"/>
+    <col min="13" max="13" width="22" customWidth="true" style="0"/>
+    <col min="14" max="14" width="22" customWidth="true" style="0"/>
+  </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" spans="1:14">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -143,6 +489,62 @@
         <v>13</v>
       </c>
     </row>
+    <row r="2" spans="1:14">
+      <c r="A2" t="s">
+        <v>14</v>
+      </c>
+      <c r="B2">
+        <v>1234567890</v>
+      </c>
+      <c r="C2" t="s">
+        <v>15</v>
+      </c>
+      <c r="D2" t="s">
+        <v>16</v>
+      </c>
+      <c r="E2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2">
+        <v>9123456789</v>
+      </c>
+      <c r="G2" t="s">
+        <v>18</v>
+      </c>
+      <c r="H2" t="s">
+        <v>19</v>
+      </c>
+      <c r="I2" t="s">
+        <v>20</v>
+      </c>
+      <c r="J2">
+        <v>15250.0</v>
+      </c>
+      <c r="K2" t="s">
+        <v>21</v>
+      </c>
+      <c r="L2" t="s">
+        <v>22</v>
+      </c>
+      <c r="M2">
+        <v>3500.0</v>
+      </c>
+      <c r="N2" t="s">
+        <v>23</v>
+      </c>
+    </row>
   </sheetData>
+  <printOptions gridLines="false" gridLinesSet="true"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1" pageOrder="downThenOver"/>
+  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
+    <oddHeader/>
+    <oddFooter/>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="0"/>
 </worksheet>
 </file>
</xml_diff>